<commit_message>
Update readme, loss simulator, input template and pool structuring overview, per WB feedback
</commit_message>
<xml_diff>
--- a/RiskPoolStructuring/PoolingTool_UploadTemplate.xlsx
+++ b/RiskPoolStructuring/PoolingTool_UploadTemplate.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="28623"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="10608"/>
   <workbookPr codeName="ThisWorkbook" defaultThemeVersion="202300"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\JamesMcIlwaine\applications\idf.finance.tool1\inst\shiny-app\Tool1\data\templates\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/stufraser/github/FinancialRiskPooling/RiskPoolStructuring/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{A275D6E8-D67A-421E-B4A6-3F373EF26C59}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{03B161B7-ECBC-8045-A47F-9606575BB543}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-110" yWindow="-110" windowWidth="25820" windowHeight="10300" activeTab="1" xr2:uid="{60C19487-0B79-41E6-A2D2-FCACF4A2B570}"/>
+    <workbookView xWindow="-120" yWindow="500" windowWidth="25820" windowHeight="10300" xr2:uid="{60C19487-0B79-41E6-A2D2-FCACF4A2B570}"/>
   </bookViews>
   <sheets>
     <sheet name="Data_Schema" sheetId="2" r:id="rId1"/>
@@ -199,12 +199,6 @@
     <t>Drought</t>
   </si>
   <si>
-    <t>Any Country from World Bank tool list (selectable from dropdown)</t>
-  </si>
-  <si>
-    <t>Any of the four perils in the World Bank tool (selectable from dropdown)</t>
-  </si>
-  <si>
     <t>Any value &gt; 0</t>
   </si>
   <si>
@@ -230,6 +224,12 @@
   </si>
   <si>
     <t>event 2</t>
+  </si>
+  <si>
+    <t>Any Country from the country list in Loss Simulator (selectable from dropdown)</t>
+  </si>
+  <si>
+    <t>Any of the four perils in the peril list in Loss Simulator (selectable from dropdown)</t>
   </si>
 </sst>
 </file>
@@ -1253,35 +1253,35 @@
     <tabColor theme="1"/>
   </sheetPr>
   <dimension ref="A1:B14"/>
-  <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
+  <sheetFormatPr baseColWidth="10" defaultColWidth="8.83203125" defaultRowHeight="15" x14ac:dyDescent="0.2"/>
   <cols>
-    <col min="1" max="1" width="19.77734375" customWidth="1"/>
-    <col min="2" max="2" width="63.77734375" customWidth="1"/>
+    <col min="1" max="1" width="19.83203125" customWidth="1"/>
+    <col min="2" max="2" width="63.83203125" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:2" x14ac:dyDescent="0.3">
+    <row r="1" spans="1:2" x14ac:dyDescent="0.2">
       <c r="A1" s="8" t="s">
+        <v>58</v>
+      </c>
+    </row>
+    <row r="2" spans="1:2" x14ac:dyDescent="0.2">
+      <c r="A2" s="3" t="s">
+        <v>59</v>
+      </c>
+      <c r="B2" s="4"/>
+    </row>
+    <row r="3" spans="1:2" x14ac:dyDescent="0.2">
+      <c r="A3" s="6" t="s">
         <v>60</v>
       </c>
-    </row>
-    <row r="2" spans="1:2" x14ac:dyDescent="0.3">
-      <c r="A2" s="3" t="s">
-        <v>61</v>
-      </c>
-      <c r="B2" s="4"/>
-    </row>
-    <row r="3" spans="1:2" x14ac:dyDescent="0.3">
-      <c r="A3" s="6" t="s">
-        <v>62</v>
-      </c>
       <c r="B3" s="7"/>
     </row>
-    <row r="5" spans="1:2" x14ac:dyDescent="0.3">
+    <row r="5" spans="1:2" x14ac:dyDescent="0.2">
       <c r="A5" s="8" t="s">
         <v>8</v>
       </c>
     </row>
-    <row r="6" spans="1:2" x14ac:dyDescent="0.3">
+    <row r="6" spans="1:2" x14ac:dyDescent="0.2">
       <c r="A6" s="13" t="s">
         <v>5</v>
       </c>
@@ -1289,7 +1289,7 @@
         <v>10</v>
       </c>
     </row>
-    <row r="7" spans="1:2" x14ac:dyDescent="0.3">
+    <row r="7" spans="1:2" x14ac:dyDescent="0.2">
       <c r="A7" s="14" t="s">
         <v>6</v>
       </c>
@@ -1297,45 +1297,45 @@
         <v>11</v>
       </c>
     </row>
-    <row r="8" spans="1:2" x14ac:dyDescent="0.3">
+    <row r="8" spans="1:2" x14ac:dyDescent="0.2">
       <c r="A8" s="14" t="s">
         <v>7</v>
       </c>
       <c r="B8" s="5" t="s">
-        <v>54</v>
-      </c>
-    </row>
-    <row r="9" spans="1:2" x14ac:dyDescent="0.3">
+        <v>63</v>
+      </c>
+    </row>
+    <row r="9" spans="1:2" x14ac:dyDescent="0.2">
       <c r="A9" s="14" t="s">
         <v>3</v>
       </c>
       <c r="B9" s="5" t="s">
-        <v>55</v>
-      </c>
-    </row>
-    <row r="10" spans="1:2" x14ac:dyDescent="0.3">
+        <v>64</v>
+      </c>
+    </row>
+    <row r="10" spans="1:2" x14ac:dyDescent="0.2">
       <c r="A10" s="15" t="s">
         <v>4</v>
       </c>
       <c r="B10" s="7" t="s">
+        <v>54</v>
+      </c>
+    </row>
+    <row r="12" spans="1:2" x14ac:dyDescent="0.2">
+      <c r="A12" s="8" t="s">
         <v>56</v>
       </c>
     </row>
-    <row r="12" spans="1:2" x14ac:dyDescent="0.3">
-      <c r="A12" s="8" t="s">
-        <v>58</v>
-      </c>
-    </row>
-    <row r="13" spans="1:2" x14ac:dyDescent="0.3">
+    <row r="13" spans="1:2" x14ac:dyDescent="0.2">
       <c r="A13" s="11"/>
       <c r="B13" s="4" t="s">
-        <v>57</v>
-      </c>
-    </row>
-    <row r="14" spans="1:2" x14ac:dyDescent="0.3">
+        <v>55</v>
+      </c>
+    </row>
+    <row r="14" spans="1:2" x14ac:dyDescent="0.2">
       <c r="A14" s="12"/>
       <c r="B14" s="7" t="s">
-        <v>59</v>
+        <v>57</v>
       </c>
     </row>
   </sheetData>
@@ -1355,16 +1355,16 @@
     <tabColor theme="5" tint="0.79998168889431442"/>
   </sheetPr>
   <dimension ref="A1:H3"/>
-  <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
+  <sheetFormatPr baseColWidth="10" defaultColWidth="8.83203125" defaultRowHeight="15" x14ac:dyDescent="0.2"/>
   <cols>
-    <col min="1" max="1" width="8.88671875" style="2"/>
-    <col min="2" max="2" width="13.21875" style="2" bestFit="1" customWidth="1"/>
+    <col min="1" max="1" width="8.83203125" style="2"/>
+    <col min="2" max="2" width="13.1640625" style="2" bestFit="1" customWidth="1"/>
     <col min="3" max="3" width="14" style="2" customWidth="1"/>
-    <col min="4" max="5" width="8.88671875" style="2"/>
-    <col min="8" max="8" width="13.109375" customWidth="1"/>
+    <col min="4" max="5" width="8.83203125" style="2"/>
+    <col min="8" max="8" width="13.1640625" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:8" ht="28.8" x14ac:dyDescent="0.3">
+    <row r="1" spans="1:8" ht="32" x14ac:dyDescent="0.2">
       <c r="A1" s="9" t="s">
         <v>5</v>
       </c>
@@ -1384,12 +1384,12 @@
         <v>9</v>
       </c>
     </row>
-    <row r="2" spans="1:8" x14ac:dyDescent="0.3">
+    <row r="2" spans="1:8" x14ac:dyDescent="0.2">
       <c r="A2" s="2">
         <v>1</v>
       </c>
       <c r="B2" s="2" t="s">
-        <v>63</v>
+        <v>61</v>
       </c>
       <c r="C2" s="2" t="s">
         <v>12</v>
@@ -1405,12 +1405,12 @@
         <v>2</v>
       </c>
     </row>
-    <row r="3" spans="1:8" x14ac:dyDescent="0.3">
+    <row r="3" spans="1:8" x14ac:dyDescent="0.2">
       <c r="A3" s="2">
         <v>2</v>
       </c>
       <c r="B3" s="2" t="s">
-        <v>64</v>
+        <v>62</v>
       </c>
       <c r="C3" s="2" t="s">
         <v>12</v>
@@ -1466,12 +1466,12 @@
     <tabColor theme="2" tint="-9.9978637043366805E-2"/>
   </sheetPr>
   <dimension ref="A1:C42"/>
-  <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
+  <sheetFormatPr baseColWidth="10" defaultColWidth="8.83203125" defaultRowHeight="15" x14ac:dyDescent="0.2"/>
   <cols>
-    <col min="1" max="1" width="25.21875" customWidth="1"/>
+    <col min="1" max="1" width="25.1640625" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:3" x14ac:dyDescent="0.3">
+    <row r="1" spans="1:3" x14ac:dyDescent="0.2">
       <c r="A1" s="1" t="s">
         <v>7</v>
       </c>
@@ -1480,7 +1480,7 @@
         <v>3</v>
       </c>
     </row>
-    <row r="2" spans="1:3" x14ac:dyDescent="0.3">
+    <row r="2" spans="1:3" x14ac:dyDescent="0.2">
       <c r="A2" t="s">
         <v>12</v>
       </c>
@@ -1488,7 +1488,7 @@
         <v>52</v>
       </c>
     </row>
-    <row r="3" spans="1:3" x14ac:dyDescent="0.3">
+    <row r="3" spans="1:3" x14ac:dyDescent="0.2">
       <c r="A3" t="s">
         <v>13</v>
       </c>
@@ -1496,7 +1496,7 @@
         <v>2</v>
       </c>
     </row>
-    <row r="4" spans="1:3" x14ac:dyDescent="0.3">
+    <row r="4" spans="1:3" x14ac:dyDescent="0.2">
       <c r="A4" t="s">
         <v>14</v>
       </c>
@@ -1504,7 +1504,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="5" spans="1:3" x14ac:dyDescent="0.3">
+    <row r="5" spans="1:3" x14ac:dyDescent="0.2">
       <c r="A5" t="s">
         <v>15</v>
       </c>
@@ -1512,187 +1512,187 @@
         <v>53</v>
       </c>
     </row>
-    <row r="6" spans="1:3" x14ac:dyDescent="0.3">
+    <row r="6" spans="1:3" x14ac:dyDescent="0.2">
       <c r="A6" t="s">
         <v>16</v>
       </c>
     </row>
-    <row r="7" spans="1:3" x14ac:dyDescent="0.3">
+    <row r="7" spans="1:3" x14ac:dyDescent="0.2">
       <c r="A7" t="s">
         <v>17</v>
       </c>
     </row>
-    <row r="8" spans="1:3" x14ac:dyDescent="0.3">
+    <row r="8" spans="1:3" x14ac:dyDescent="0.2">
       <c r="A8" t="s">
         <v>18</v>
       </c>
     </row>
-    <row r="9" spans="1:3" x14ac:dyDescent="0.3">
+    <row r="9" spans="1:3" x14ac:dyDescent="0.2">
       <c r="A9" t="s">
         <v>19</v>
       </c>
     </row>
-    <row r="10" spans="1:3" x14ac:dyDescent="0.3">
+    <row r="10" spans="1:3" x14ac:dyDescent="0.2">
       <c r="A10" t="s">
         <v>20</v>
       </c>
     </row>
-    <row r="11" spans="1:3" x14ac:dyDescent="0.3">
+    <row r="11" spans="1:3" x14ac:dyDescent="0.2">
       <c r="A11" t="s">
         <v>21</v>
       </c>
     </row>
-    <row r="12" spans="1:3" x14ac:dyDescent="0.3">
+    <row r="12" spans="1:3" x14ac:dyDescent="0.2">
       <c r="A12" t="s">
         <v>22</v>
       </c>
     </row>
-    <row r="13" spans="1:3" x14ac:dyDescent="0.3">
+    <row r="13" spans="1:3" x14ac:dyDescent="0.2">
       <c r="A13" t="s">
         <v>23</v>
       </c>
     </row>
-    <row r="14" spans="1:3" x14ac:dyDescent="0.3">
+    <row r="14" spans="1:3" x14ac:dyDescent="0.2">
       <c r="A14" t="s">
         <v>24</v>
       </c>
     </row>
-    <row r="15" spans="1:3" x14ac:dyDescent="0.3">
+    <row r="15" spans="1:3" x14ac:dyDescent="0.2">
       <c r="A15" t="s">
         <v>25</v>
       </c>
     </row>
-    <row r="16" spans="1:3" x14ac:dyDescent="0.3">
+    <row r="16" spans="1:3" x14ac:dyDescent="0.2">
       <c r="A16" t="s">
         <v>26</v>
       </c>
     </row>
-    <row r="17" spans="1:1" x14ac:dyDescent="0.3">
+    <row r="17" spans="1:1" x14ac:dyDescent="0.2">
       <c r="A17" t="s">
         <v>27</v>
       </c>
     </row>
-    <row r="18" spans="1:1" x14ac:dyDescent="0.3">
+    <row r="18" spans="1:1" x14ac:dyDescent="0.2">
       <c r="A18" t="s">
         <v>28</v>
       </c>
     </row>
-    <row r="19" spans="1:1" x14ac:dyDescent="0.3">
+    <row r="19" spans="1:1" x14ac:dyDescent="0.2">
       <c r="A19" t="s">
         <v>29</v>
       </c>
     </row>
-    <row r="20" spans="1:1" x14ac:dyDescent="0.3">
+    <row r="20" spans="1:1" x14ac:dyDescent="0.2">
       <c r="A20" t="s">
         <v>30</v>
       </c>
     </row>
-    <row r="21" spans="1:1" x14ac:dyDescent="0.3">
+    <row r="21" spans="1:1" x14ac:dyDescent="0.2">
       <c r="A21" t="s">
         <v>31</v>
       </c>
     </row>
-    <row r="22" spans="1:1" x14ac:dyDescent="0.3">
+    <row r="22" spans="1:1" x14ac:dyDescent="0.2">
       <c r="A22" t="s">
         <v>32</v>
       </c>
     </row>
-    <row r="23" spans="1:1" x14ac:dyDescent="0.3">
+    <row r="23" spans="1:1" x14ac:dyDescent="0.2">
       <c r="A23" t="s">
         <v>33</v>
       </c>
     </row>
-    <row r="24" spans="1:1" x14ac:dyDescent="0.3">
+    <row r="24" spans="1:1" x14ac:dyDescent="0.2">
       <c r="A24" t="s">
         <v>34</v>
       </c>
     </row>
-    <row r="25" spans="1:1" x14ac:dyDescent="0.3">
+    <row r="25" spans="1:1" x14ac:dyDescent="0.2">
       <c r="A25" t="s">
         <v>35</v>
       </c>
     </row>
-    <row r="26" spans="1:1" x14ac:dyDescent="0.3">
+    <row r="26" spans="1:1" x14ac:dyDescent="0.2">
       <c r="A26" t="s">
         <v>36</v>
       </c>
     </row>
-    <row r="27" spans="1:1" x14ac:dyDescent="0.3">
+    <row r="27" spans="1:1" x14ac:dyDescent="0.2">
       <c r="A27" t="s">
         <v>37</v>
       </c>
     </row>
-    <row r="28" spans="1:1" x14ac:dyDescent="0.3">
+    <row r="28" spans="1:1" x14ac:dyDescent="0.2">
       <c r="A28" t="s">
         <v>38</v>
       </c>
     </row>
-    <row r="29" spans="1:1" x14ac:dyDescent="0.3">
+    <row r="29" spans="1:1" x14ac:dyDescent="0.2">
       <c r="A29" t="s">
         <v>39</v>
       </c>
     </row>
-    <row r="30" spans="1:1" x14ac:dyDescent="0.3">
+    <row r="30" spans="1:1" x14ac:dyDescent="0.2">
       <c r="A30" t="s">
         <v>40</v>
       </c>
     </row>
-    <row r="31" spans="1:1" x14ac:dyDescent="0.3">
+    <row r="31" spans="1:1" x14ac:dyDescent="0.2">
       <c r="A31" t="s">
         <v>41</v>
       </c>
     </row>
-    <row r="32" spans="1:1" x14ac:dyDescent="0.3">
+    <row r="32" spans="1:1" x14ac:dyDescent="0.2">
       <c r="A32" t="s">
         <v>42</v>
       </c>
     </row>
-    <row r="33" spans="1:1" x14ac:dyDescent="0.3">
+    <row r="33" spans="1:1" x14ac:dyDescent="0.2">
       <c r="A33" t="s">
         <v>43</v>
       </c>
     </row>
-    <row r="34" spans="1:1" x14ac:dyDescent="0.3">
+    <row r="34" spans="1:1" x14ac:dyDescent="0.2">
       <c r="A34" t="s">
         <v>44</v>
       </c>
     </row>
-    <row r="35" spans="1:1" x14ac:dyDescent="0.3">
+    <row r="35" spans="1:1" x14ac:dyDescent="0.2">
       <c r="A35" t="s">
         <v>0</v>
       </c>
     </row>
-    <row r="36" spans="1:1" x14ac:dyDescent="0.3">
+    <row r="36" spans="1:1" x14ac:dyDescent="0.2">
       <c r="A36" t="s">
         <v>45</v>
       </c>
     </row>
-    <row r="37" spans="1:1" x14ac:dyDescent="0.3">
+    <row r="37" spans="1:1" x14ac:dyDescent="0.2">
       <c r="A37" t="s">
         <v>46</v>
       </c>
     </row>
-    <row r="38" spans="1:1" x14ac:dyDescent="0.3">
+    <row r="38" spans="1:1" x14ac:dyDescent="0.2">
       <c r="A38" t="s">
         <v>47</v>
       </c>
     </row>
-    <row r="39" spans="1:1" x14ac:dyDescent="0.3">
+    <row r="39" spans="1:1" x14ac:dyDescent="0.2">
       <c r="A39" t="s">
         <v>48</v>
       </c>
     </row>
-    <row r="40" spans="1:1" x14ac:dyDescent="0.3">
+    <row r="40" spans="1:1" x14ac:dyDescent="0.2">
       <c r="A40" t="s">
         <v>49</v>
       </c>
     </row>
-    <row r="41" spans="1:1" x14ac:dyDescent="0.3">
+    <row r="41" spans="1:1" x14ac:dyDescent="0.2">
       <c r="A41" t="s">
         <v>50</v>
       </c>
     </row>
-    <row r="42" spans="1:1" x14ac:dyDescent="0.3">
+    <row r="42" spans="1:1" x14ac:dyDescent="0.2">
       <c r="A42" t="s">
         <v>51</v>
       </c>

</xml_diff>

<commit_message>
Updating app.R and global.R per WB feedback, update custom.css to IDF branding
</commit_message>
<xml_diff>
--- a/RiskPoolStructuring/PoolingTool_UploadTemplate.xlsx
+++ b/RiskPoolStructuring/PoolingTool_UploadTemplate.xlsx
@@ -5,10 +5,10 @@
   <workbookPr codeName="ThisWorkbook" defaultThemeVersion="202300"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/stufraser/github/FinancialRiskPooling/RiskPoolStructuring/"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/stufraser/github/DisasterRiskPooling/RiskPoolStructuring/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{03B161B7-ECBC-8045-A47F-9606575BB543}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{16A14FFD-CF42-DB41-8E74-75EDCE78FAB1}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-120" yWindow="500" windowWidth="25820" windowHeight="10300" xr2:uid="{60C19487-0B79-41E6-A2D2-FCACF4A2B570}"/>
   </bookViews>
@@ -217,9 +217,6 @@
     <t>The purpose of this file is to enable you to upload modelled loss output or historical  loss output</t>
   </si>
   <si>
-    <t>into tool1 for further use in the modelling.</t>
-  </si>
-  <si>
     <t>event 1</t>
   </si>
   <si>
@@ -230,6 +227,9 @@
   </si>
   <si>
     <t>Any of the four perils in the peril list in Loss Simulator (selectable from dropdown)</t>
+  </si>
+  <si>
+    <t>into the Loss Simulator for further use in the modelling.</t>
   </si>
 </sst>
 </file>
@@ -1272,7 +1272,7 @@
     </row>
     <row r="3" spans="1:2" x14ac:dyDescent="0.2">
       <c r="A3" s="6" t="s">
-        <v>60</v>
+        <v>64</v>
       </c>
       <c r="B3" s="7"/>
     </row>
@@ -1302,7 +1302,7 @@
         <v>7</v>
       </c>
       <c r="B8" s="5" t="s">
-        <v>63</v>
+        <v>62</v>
       </c>
     </row>
     <row r="9" spans="1:2" x14ac:dyDescent="0.2">
@@ -1310,7 +1310,7 @@
         <v>3</v>
       </c>
       <c r="B9" s="5" t="s">
-        <v>64</v>
+        <v>63</v>
       </c>
     </row>
     <row r="10" spans="1:2" x14ac:dyDescent="0.2">
@@ -1389,7 +1389,7 @@
         <v>1</v>
       </c>
       <c r="B2" s="2" t="s">
-        <v>61</v>
+        <v>60</v>
       </c>
       <c r="C2" s="2" t="s">
         <v>12</v>
@@ -1410,7 +1410,7 @@
         <v>2</v>
       </c>
       <c r="B3" s="2" t="s">
-        <v>62</v>
+        <v>61</v>
       </c>
       <c r="C3" s="2" t="s">
         <v>12</v>

</xml_diff>